<commit_message>
Vulnerable groups extract 2026-07-08T02:50:46Z
</commit_message>
<xml_diff>
--- a/docs/vulnerable-groups.xlsx
+++ b/docs/vulnerable-groups.xlsx
@@ -409,7 +409,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Generated: 2026-07-08 01:48:48 UTC</v>
+        <v>Generated: 2026-07-08 02:50:46 UTC</v>
       </c>
     </row>
     <row r="4">
@@ -449,17 +449,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Disability (standard WG): 0</v>
+        <v>Disability (standard WG): 304</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Disability (broader): 0</v>
+        <v>Disability (broader): 1678</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Migration merged: 2</v>
+        <v>Migration merged: 3</v>
       </c>
     </row>
     <row r="17">
@@ -469,7 +469,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">  NONE - detection failed, check survey structure</v>
+        <v xml:space="preserve">  289909840: Does your child have difficulty seeing, even if wearing glasses?, Does your child have dif</v>
       </c>
     </row>
   </sheetData>
@@ -481,7 +481,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D34"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -514,7 +514,7 @@
         <v/>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3">
@@ -522,32 +522,452 @@
         <v/>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>District</v>
       </c>
       <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>SP Tengah</v>
+      </c>
+      <c r="D3">
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>District</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Timur Laut</v>
+      </c>
+      <c r="D4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v>District</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Barat Daya</v>
+      </c>
+      <c r="D5">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v>District</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SP Utara</v>
+      </c>
+      <c r="D6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v>District</v>
+      </c>
+      <c r="C7" t="str">
+        <v>SP Selatan</v>
+      </c>
+      <c r="D7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v>District</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D9">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Female</v>
+      </c>
+      <c r="D10">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C11" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="D11">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C12" t="str">
+        <v>13-16</v>
+      </c>
+      <c r="D12">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C13" t="str">
+        <v>17</v>
+      </c>
+      <c r="D13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C14" t="str">
+        <v>M40</v>
+      </c>
+      <c r="D14">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C15" t="str">
+        <v>T20</v>
+      </c>
+      <c r="D15">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C16" t="str">
+        <v>B40</v>
+      </c>
+      <c r="D16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="D17">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Disability - broader (some difficulty+)</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B19" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4">
-        <v>0</v>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19">
+        <v>1678</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v>District</v>
+      </c>
+      <c r="C20" t="str">
+        <v>SP Tengah</v>
+      </c>
+      <c r="D20">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+      <c r="B21" t="str">
+        <v>District</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Timur Laut</v>
+      </c>
+      <c r="D21">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+      <c r="B22" t="str">
+        <v>District</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Barat Daya</v>
+      </c>
+      <c r="D22">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v/>
+      </c>
+      <c r="B23" t="str">
+        <v>District</v>
+      </c>
+      <c r="C23" t="str">
+        <v>SP Utara</v>
+      </c>
+      <c r="D23">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+      <c r="B24" t="str">
+        <v>District</v>
+      </c>
+      <c r="C24" t="str">
+        <v>SP Selatan</v>
+      </c>
+      <c r="D24">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v>District</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Female</v>
+      </c>
+      <c r="D26">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D27">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v/>
+      </c>
+      <c r="B28" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C28" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="D28">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+      <c r="B29" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C29" t="str">
+        <v>13-16</v>
+      </c>
+      <c r="D29">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v>Age</v>
+      </c>
+      <c r="C30" t="str">
+        <v>17</v>
+      </c>
+      <c r="D30">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v/>
+      </c>
+      <c r="B31" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C31" t="str">
+        <v>M40</v>
+      </c>
+      <c r="D31">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+      <c r="B32" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C32" t="str">
+        <v>T20</v>
+      </c>
+      <c r="D32">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v/>
+      </c>
+      <c r="B33" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C33" t="str">
+        <v>B40</v>
+      </c>
+      <c r="D33">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="D34">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -811,7 +1231,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>YES</v>
       </c>
     </row>
     <row r="24">
@@ -922,7 +1342,7 @@
         <v/>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -936,7 +1356,7 @@
         <v>Barat Daya</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">

</xml_diff>